<commit_message>
Add 2026 Year-1 financial model, expand nav index with sub-section anchors, fix warranty wording
- Split Finance/Accounting into 3.5.1 (2026 Year 1, monthly) and 3.5.2 (2027 three scenarios), properly cross-referenced and numbered
- Expanded the Index dropdown nav on every page with chapter/sub-section anchors and a "View Full Index" link
- Fixed a leftover "supervisor" reference inconsistent with the Friendly Customer Service warranty's store-manager-only approval
- Updated IFE matrix, campaign plan and 2027 financial statement workbooks

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Estados_Financieros_Doner_Street_2027.xlsx
+++ b/Estados_Financieros_Doner_Street_2027.xlsx
@@ -1086,7 +1086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1102,6 +1102,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1141,10 +1142,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>180332099</v>
+        <v>196344259</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>409434835</v>
+        <v>430648125</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>0</v>
@@ -1153,489 +1154,457 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Cuentas por cobrar</t>
+          <t xml:space="preserve">    Inventarios</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>10512160</v>
+        <v>5000000</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>15713290</v>
+        <v>5000000</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>6108875</v>
+        <v>5000000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Inventarios</t>
+          <t xml:space="preserve">    Anticipos e impuestos a favor</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Total activo corriente</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>201344259</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>435648125</v>
+      </c>
+      <c r="D8" s="8" t="n">
         <v>5000000</v>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>5000000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Anticipos e impuestos a favor</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Gastos pagados por anticipado</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>5500000</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>5500000</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>5500000</v>
-      </c>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVO NO CORRIENTE</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Total activo corriente</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="n">
-        <v>201344259</v>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>435648125</v>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>16608875</v>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    PP&amp;E (bruto)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>85000000</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>85000000</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>85000000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>ACTIVO NO CORRIENTE</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    (-) Depreciación acumulada</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>17000000</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    PP&amp;E (bruto)</t>
+          <t xml:space="preserve">    PP&amp;E, neto</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>85000000</v>
+        <v>68000000</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>85000000</v>
+        <v>68000000</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>85000000</v>
+        <v>68000000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (-) Depreciación acumulada</t>
+          <t xml:space="preserve">    Intangibles, neto</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>17000000</v>
+        <v>0</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>17000000</v>
+        <v>0</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>17000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    PP&amp;E, neto</t>
+          <t xml:space="preserve">    Inversiones LP</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Total activo no corriente</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
         <v>68000000</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C15" s="8" t="n">
         <v>68000000</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D15" s="8" t="n">
         <v>68000000</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Intangibles, neto</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Inversiones LP</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>0</v>
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL ACTIVO</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>269344259</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>503648125</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>73000000</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Total activo no corriente</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>68000000</v>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>68000000</v>
-      </c>
-      <c r="D17" s="8" t="n">
-        <v>68000000</v>
-      </c>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>PASIVO CORRIENTE</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL ACTIVO</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="n">
-        <v>269344259</v>
-      </c>
-      <c r="C18" s="9" t="n">
-        <v>503648125</v>
-      </c>
-      <c r="D18" s="9" t="n">
-        <v>84608875</v>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Proveedores</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>31046640</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>46291592</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>18169536</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>PASIVO CORRIENTE</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Obligaciones financieras CP (sobregiro)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>21631025</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Proveedores</t>
+          <t xml:space="preserve">    Nómina por pagar y prestaciones</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>31046640</v>
+        <v>30942000</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>46291592</v>
+        <v>33048000</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>18169536</v>
+        <v>30942000</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Obligaciones financieras CP (sobregiro)</t>
+          <t xml:space="preserve">    Seguridad social y parafiscales</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>0</v>
+        <v>3915500</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>0</v>
+        <v>4182000</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>33239900</v>
+        <v>3915500</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Nómina por pagar y prestaciones</t>
+          <t xml:space="preserve">    Impuestos por pagar</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>30942000</v>
+        <v>31277179</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>33048000</v>
+        <v>110339451</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>30942000</v>
+        <v>6262097</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Seguridad social y parafiscales</t>
+          <t xml:space="preserve">    Otras cuentas por pagar</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>3915500</v>
+        <v>3500000</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>4182000</v>
+        <v>3500000</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>3915500</v>
+        <v>3500000</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Impuestos por pagar</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>31277179</v>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>110339451</v>
-      </c>
-      <c r="D24" s="5" t="n">
-        <v>6262097</v>
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Total pasivo corriente</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>100681319</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>197361043</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>84420158</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Otras cuentas por pagar</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>3500000</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>3500000</v>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>3500000</v>
-      </c>
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>PASIVO NO CORRIENTE</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Total pasivo corriente</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Obligaciones financieras LP</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Préstamos de socios</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL PASIVO</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="n">
         <v>100681319</v>
       </c>
-      <c r="C26" s="8" t="n">
+      <c r="C28" s="8" t="n">
         <v>197361043</v>
       </c>
-      <c r="D26" s="8" t="n">
-        <v>96029033</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>PASIVO NO CORRIENTE</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Obligaciones financieras LP</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="5" t="n">
-        <v>0</v>
+      <c r="D28" s="8" t="n">
+        <v>84420158</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Préstamos de socios</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>0</v>
-      </c>
-      <c r="C29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>PATRIMONIO</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL PASIVO</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="n">
-        <v>100681319</v>
-      </c>
-      <c r="C30" s="8" t="n">
-        <v>197361043</v>
-      </c>
-      <c r="D30" s="8" t="n">
-        <v>96029033</v>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Capital social</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>130000000</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>130000000</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>130000000</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>PATRIMONIO</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Reserva legal</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Capital social</t>
+          <t xml:space="preserve">    Utilidades retenidas anteriores</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>130000000</v>
+        <v>0</v>
       </c>
       <c r="C32" s="5" t="n">
-        <v>130000000</v>
+        <v>0</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>130000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Reserva legal</t>
+          <t xml:space="preserve">    Utilidad del ejercicio</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>0</v>
+        <v>38662940</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>0</v>
+        <v>176287082</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>0</v>
+        <v>-141420158</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Utilidades retenidas anteriores</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="5" t="n">
-        <v>0</v>
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL PATRIMONIO</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="n">
+        <v>168662940</v>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>306287082</v>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>-11420158</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Utilidad del ejercicio</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>38662940</v>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>176287082</v>
-      </c>
-      <c r="D35" s="5" t="n">
-        <v>-141420158</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL PATRIMONIO</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="n">
-        <v>168662940</v>
-      </c>
-      <c r="C36" s="9" t="n">
-        <v>306287082</v>
-      </c>
-      <c r="D36" s="9" t="n">
-        <v>-11420158</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>TOTAL PASIVO + PATRIMONIO</t>
         </is>
       </c>
-      <c r="B37" s="8" t="n">
+      <c r="B35" s="8" t="n">
         <v>269344259</v>
       </c>
-      <c r="C37" s="8" t="n">
+      <c r="C35" s="8" t="n">
         <v>503648125</v>
       </c>
-      <c r="D37" s="8" t="n">
-        <v>84608875</v>
+      <c r="D35" s="8" t="n">
+        <v>73000000</v>
       </c>
     </row>
   </sheetData>
@@ -1649,7 +1618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1665,6 +1634,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1732,341 +1702,309 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (-) Aumento en CxC</t>
+          <t xml:space="preserve">    (+) Aumento en proveedores</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>10512160</v>
+        <v>31046640</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>15713290</v>
+        <v>46291592</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>6108875</v>
+        <v>18169536</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (-) Aumento en gastos pag. anticipado</t>
+          <t xml:space="preserve">    (+) Aumento en nómina por pagar</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5500000</v>
+        <v>30942000</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>5500000</v>
+        <v>33048000</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>5500000</v>
+        <v>30942000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (+) Aumento en proveedores</t>
+          <t xml:space="preserve">    (+) Aumento en seg. social/parafiscales</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>31046640</v>
+        <v>3915500</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>46291592</v>
+        <v>4182000</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>18169536</v>
+        <v>3915500</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (+) Aumento en nómina por pagar</t>
+          <t xml:space="preserve">    (+) Aumento en impuestos por pagar</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>30942000</v>
+        <v>31277179</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>33048000</v>
+        <v>110339451</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>30942000</v>
+        <v>6262097</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (+) Aumento en seg. social/parafiscales</t>
+          <t xml:space="preserve">    (+) Aumento en otras CxP</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>3915500</v>
+        <v>3500000</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>4182000</v>
+        <v>3500000</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>3915500</v>
+        <v>3500000</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    (+) Aumento en impuestos por pagar</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>31277179</v>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>110339451</v>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>6262097</v>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Efectivo neto de operación</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>156344259</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>390648125</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>-61631025</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    (+) Aumento en otras CxP</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>3500000</v>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>3500000</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>3500000</v>
-      </c>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVIDADES DE INVERSIÓN</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Efectivo neto de operación</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="n">
-        <v>140332099</v>
-      </c>
-      <c r="C14" s="9" t="n">
-        <v>369434835</v>
-      </c>
-      <c r="D14" s="11" t="n">
-        <v>-73239900</v>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Compra de PP&amp;E</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>-85000000</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>-85000000</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>-85000000</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>ACTIVIDADES DE INVERSIÓN</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Compra de inventario de apertura</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>-5000000</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>-5000000</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>-5000000</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Compra de PP&amp;E</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>-85000000</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>-85000000</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>-85000000</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Venta de activos</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Compra de inventario de apertura</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>-5000000</v>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>-5000000</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>-5000000</v>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Efectivo neto de inversión</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>-90000000</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>-90000000</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>-90000000</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Venta de activos</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVIDADES DE FINANCIACIÓN</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Efectivo neto de inversión</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="n">
-        <v>-90000000</v>
-      </c>
-      <c r="C19" s="8" t="n">
-        <v>-90000000</v>
-      </c>
-      <c r="D19" s="8" t="n">
-        <v>-90000000</v>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Aporte de capital social</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>130000000</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>130000000</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>130000000</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>ACTIVIDADES DE FINANCIACIÓN</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Préstamos recibidos</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Aporte de capital social</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Abonos a capital de créditos</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Dividendos pagados</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Efectivo neto de financiación</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="n">
         <v>130000000</v>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C23" s="8" t="n">
         <v>130000000</v>
       </c>
-      <c r="D21" s="5" t="n">
+      <c r="D23" s="8" t="n">
         <v>130000000</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Préstamos recibidos</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Abonos a capital de créditos</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0</v>
-      </c>
-    </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Dividendos pagados</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="5" t="n">
-        <v>0</v>
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Flujo neto del periodo</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>196344259</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>430648125</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>-21631025</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Efectivo neto de financiación</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="n">
-        <v>130000000</v>
-      </c>
-      <c r="C25" s="8" t="n">
-        <v>130000000</v>
-      </c>
-      <c r="D25" s="8" t="n">
-        <v>130000000</v>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Saldo inicial de efectivo</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Flujo neto del periodo</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n">
-        <v>180332099</v>
-      </c>
-      <c r="C26" s="8" t="n">
-        <v>409434835</v>
-      </c>
-      <c r="D26" s="8" t="n">
-        <v>-33239900</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Saldo inicial de efectivo</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
           <t>Saldo final de efectivo</t>
         </is>
       </c>
-      <c r="B28" s="9" t="n">
-        <v>180332099</v>
-      </c>
-      <c r="C28" s="9" t="n">
-        <v>409434835</v>
-      </c>
-      <c r="D28" s="11" t="n">
-        <v>-33239900</v>
+      <c r="B26" s="9" t="n">
+        <v>196344259</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>430648125</v>
+      </c>
+      <c r="D26" s="11" t="n">
+        <v>-21631025</v>
       </c>
     </row>
   </sheetData>
@@ -2096,6 +2034,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2173,13 +2112,13 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>180332099</v>
+        <v>196344259</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>409434835</v>
+        <v>430648125</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>-33239900</v>
+        <v>-21631025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>